<commit_message>
Guardar estado pendiente antes de reestructurar (Docker app + definicion de experimento)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Definir experimento.xlsx
+++ b/Definir experimento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\06Docencia\01Dictado de cursos\08PECD\02Aprendizaje Supervisado\06ML\ml-supervisado-uni\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4809C5E6-C982-4412-B58B-D71DEC741E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC2C186-7E6D-4941-BC14-267F3F2FC677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4335" yWindow="1230" windowWidth="15825" windowHeight="13770" xr2:uid="{337C9C22-3E5F-4FC9-9455-B210786D96EF}"/>
+    <workbookView xWindow="-120" yWindow="16080" windowWidth="19440" windowHeight="14880" xr2:uid="{337C9C22-3E5F-4FC9-9455-B210786D96EF}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="42">
   <si>
     <t xml:space="preserve">18 meses cosecha </t>
   </si>
@@ -141,6 +141,27 @@
   </si>
   <si>
     <t>df testing</t>
+  </si>
+  <si>
+    <t>nuevos clientes, nuevos segmentos</t>
+  </si>
+  <si>
+    <t>valores atípicos, nulos</t>
+  </si>
+  <si>
+    <t>Hipótesis</t>
+  </si>
+  <si>
+    <t>1: modelar con 6 meses de historia, incluyendo</t>
+  </si>
+  <si>
+    <t>train_test_split</t>
+  </si>
+  <si>
+    <t>Análisis médicos</t>
+  </si>
+  <si>
+    <t>Optimización</t>
   </si>
 </sst>
 </file>
@@ -227,7 +248,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -235,11 +256,73 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color theme="8"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="8"/>
+      </right>
+      <top style="medium">
+        <color theme="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="8"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -248,9 +331,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -585,18 +674,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7D0F36-DD77-4020-A298-9A4AD189F242}">
-  <dimension ref="A1:AI48"/>
+  <dimension ref="A1:AJ48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="5.69140625" customWidth="1"/>
-    <col min="2" max="2" width="13.07421875" customWidth="1"/>
+    <col min="2" max="2" width="13.61328125" customWidth="1"/>
     <col min="3" max="3" width="5.3828125" customWidth="1"/>
     <col min="4" max="29" width="4.69140625" customWidth="1"/>
     <col min="30" max="33" width="4.61328125" customWidth="1"/>
     <col min="34" max="34" width="5.15234375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.4">
       <c r="E1" s="3"/>
       <c r="F1" t="s">
         <v>1</v>
@@ -609,8 +698,71 @@
       <c r="S1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.4">
+      <c r="AJ1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="U2">
+        <f ca="1">RANDBETWEEN(3,4)</f>
+        <v>4</v>
+      </c>
+      <c r="V2">
+        <f t="shared" ref="V2:AG2" ca="1" si="0">RANDBETWEEN(3,4)</f>
+        <v>4</v>
+      </c>
+      <c r="W2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="X2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="Y2">
+        <f t="shared" ca="1" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="Z2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="AA2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="AB2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="AC2">
+        <f t="shared" ca="1" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="AD2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="AE2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="AF2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="AG2">
+        <f t="shared" ca="1" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="AH2">
+        <v>6</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.4">
       <c r="D3">
         <v>2307</v>
       </c>
@@ -705,12 +857,15 @@
         <v>2601</v>
       </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>30</v>
       </c>
       <c r="C4">
         <v>2512</v>
+      </c>
+      <c r="D4">
+        <v>50</v>
       </c>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
@@ -727,15 +882,19 @@
       <c r="AG4" s="1"/>
       <c r="AH4" s="2"/>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <v>2511</v>
+      </c>
+      <c r="D5">
+        <f t="shared" ref="D5:D8" ca="1" si="1">+RANDBETWEEN(65,68)</f>
+        <v>68</v>
       </c>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
@@ -752,16 +911,20 @@
       <c r="AF5" s="1"/>
       <c r="AG5" s="2"/>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <f>+C5-1</f>
         <v>2510</v>
+      </c>
+      <c r="D6">
+        <f t="shared" ca="1" si="1"/>
+        <v>65</v>
       </c>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
@@ -778,16 +941,20 @@
       <c r="AE6" s="1"/>
       <c r="AF6" s="2"/>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:36" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="10">
-        <f t="shared" ref="C7:C15" si="0">+C6-1</f>
+      <c r="C7" s="8">
+        <f t="shared" ref="C7:C15" si="2">+C6-1</f>
         <v>2509</v>
+      </c>
+      <c r="D7">
+        <f t="shared" ca="1" si="1"/>
+        <v>67</v>
       </c>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
@@ -804,13 +971,17 @@
       <c r="AD7" s="1"/>
       <c r="AE7" s="2"/>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B8" s="8" t="s">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="8">
-        <f t="shared" si="0"/>
+      <c r="C8" s="10">
+        <f t="shared" si="2"/>
         <v>2508</v>
+      </c>
+      <c r="D8">
+        <f ca="1">+RANDBETWEEN(65,68)</f>
+        <v>66</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
@@ -827,13 +998,17 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="2"/>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B9" s="8" t="s">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B9" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="8">
-        <f t="shared" si="0"/>
+      <c r="C9" s="12">
+        <f t="shared" si="2"/>
         <v>2507</v>
+      </c>
+      <c r="D9">
+        <f t="shared" ref="D9:D21" ca="1" si="3">+RANDBETWEEN(65,68)</f>
+        <v>67</v>
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
@@ -850,13 +1025,17 @@
       <c r="AB9" s="1"/>
       <c r="AC9" s="2"/>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B10" s="8" t="s">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B10" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="8">
-        <f t="shared" si="0"/>
+      <c r="C10" s="12">
+        <f t="shared" si="2"/>
         <v>2506</v>
+      </c>
+      <c r="D10">
+        <f t="shared" ca="1" si="3"/>
+        <v>66</v>
       </c>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -873,13 +1052,20 @@
       <c r="AA10" s="1"/>
       <c r="AB10" s="2"/>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B11" s="9" t="s">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="9">
-        <f t="shared" si="0"/>
+      <c r="C11" s="14">
+        <f t="shared" si="2"/>
         <v>2505</v>
+      </c>
+      <c r="D11">
+        <f t="shared" ca="1" si="3"/>
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
       </c>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
@@ -899,13 +1085,20 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B12" s="9" t="s">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B12" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="9">
-        <f t="shared" si="0"/>
+      <c r="C12" s="14">
+        <f t="shared" si="2"/>
         <v>2504</v>
+      </c>
+      <c r="D12">
+        <f t="shared" ca="1" si="3"/>
+        <v>65</v>
+      </c>
+      <c r="E12" t="s">
+        <v>39</v>
       </c>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
@@ -925,13 +1118,20 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B13" s="9" t="s">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B13" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="9">
-        <f t="shared" si="0"/>
+      <c r="C13" s="14">
+        <f t="shared" si="2"/>
         <v>2503</v>
+      </c>
+      <c r="D13">
+        <f t="shared" ca="1" si="3"/>
+        <v>65</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
       </c>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
@@ -955,13 +1155,20 @@
       <c r="AG13" s="7"/>
       <c r="AH13" s="7"/>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B14" s="9" t="s">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B14" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="9">
-        <f t="shared" si="0"/>
+      <c r="C14" s="14">
+        <f t="shared" si="2"/>
         <v>2502</v>
+      </c>
+      <c r="D14">
+        <f t="shared" ca="1" si="3"/>
+        <v>68</v>
+      </c>
+      <c r="E14" t="s">
+        <v>39</v>
       </c>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
@@ -978,13 +1185,20 @@
       <c r="W14" s="1"/>
       <c r="X14" s="2"/>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B15" s="9" t="s">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B15" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="9">
-        <f t="shared" si="0"/>
+      <c r="C15" s="14">
+        <f t="shared" si="2"/>
         <v>2501</v>
+      </c>
+      <c r="D15">
+        <f t="shared" ca="1" si="3"/>
+        <v>66</v>
+      </c>
+      <c r="E15" t="s">
+        <v>39</v>
       </c>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
@@ -1004,13 +1218,20 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="B16" s="9" t="s">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="B16" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="14">
         <f>+C4-100</f>
         <v>2412</v>
+      </c>
+      <c r="D16">
+        <f t="shared" ca="1" si="3"/>
+        <v>67</v>
+      </c>
+      <c r="E16" t="s">
+        <v>39</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
@@ -1031,12 +1252,19 @@
       </c>
     </row>
     <row r="17" spans="2:35" x14ac:dyDescent="0.4">
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="9">
-        <f t="shared" ref="C17:C21" si="1">+C5-100</f>
+      <c r="C17" s="14">
+        <f t="shared" ref="C17:C21" si="4">+C5-100</f>
         <v>2411</v>
+      </c>
+      <c r="D17">
+        <f t="shared" ca="1" si="3"/>
+        <v>66</v>
+      </c>
+      <c r="E17" t="s">
+        <v>39</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -1057,12 +1285,19 @@
       </c>
     </row>
     <row r="18" spans="2:35" x14ac:dyDescent="0.4">
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="9">
-        <f t="shared" si="1"/>
+      <c r="C18" s="14">
+        <f t="shared" si="4"/>
         <v>2410</v>
+      </c>
+      <c r="D18">
+        <f t="shared" ca="1" si="3"/>
+        <v>68</v>
+      </c>
+      <c r="E18" t="s">
+        <v>39</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
@@ -1086,12 +1321,19 @@
       </c>
     </row>
     <row r="19" spans="2:35" x14ac:dyDescent="0.4">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="9">
-        <f t="shared" si="1"/>
+      <c r="C19" s="14">
+        <f t="shared" si="4"/>
         <v>2409</v>
+      </c>
+      <c r="D19">
+        <f t="shared" ca="1" si="3"/>
+        <v>67</v>
+      </c>
+      <c r="E19" t="s">
+        <v>39</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -1118,14 +1360,20 @@
       </c>
     </row>
     <row r="20" spans="2:35" x14ac:dyDescent="0.4">
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="9">
-        <f t="shared" si="1"/>
+      <c r="C20" s="14">
+        <f t="shared" si="4"/>
         <v>2408</v>
       </c>
-      <c r="E20" s="3"/>
+      <c r="D20">
+        <f t="shared" ca="1" si="3"/>
+        <v>67</v>
+      </c>
+      <c r="E20" t="s">
+        <v>39</v>
+      </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
@@ -1149,16 +1397,21 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="2:35" x14ac:dyDescent="0.4">
-      <c r="B21" s="9" t="s">
+    <row r="21" spans="2:35" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B21" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="9">
-        <f t="shared" si="1"/>
+      <c r="C21" s="16">
+        <f t="shared" si="4"/>
         <v>2407</v>
       </c>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
+      <c r="D21">
+        <f t="shared" ca="1" si="3"/>
+        <v>67</v>
+      </c>
+      <c r="E21" t="s">
+        <v>39</v>
+      </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
@@ -1196,6 +1449,9 @@
       </c>
     </row>
     <row r="23" spans="2:35" x14ac:dyDescent="0.4">
+      <c r="R23" t="s">
+        <v>37</v>
+      </c>
       <c r="AC23">
         <v>2025</v>
       </c>
@@ -1207,6 +1463,9 @@
       </c>
     </row>
     <row r="24" spans="2:35" x14ac:dyDescent="0.4">
+      <c r="R24" t="s">
+        <v>38</v>
+      </c>
       <c r="AC24">
         <v>2022</v>
       </c>
@@ -1229,11 +1488,19 @@
       </c>
     </row>
     <row r="26" spans="2:35" x14ac:dyDescent="0.4">
+      <c r="B26" t="s">
+        <v>40</v>
+      </c>
       <c r="AD26" s="4" t="s">
         <v>28</v>
       </c>
       <c r="AI26" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="2:35" x14ac:dyDescent="0.4">
+      <c r="B27" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="2:35" x14ac:dyDescent="0.4">

</xml_diff>